<commit_message>
Add Tohto divisions to rating site
</commit_message>
<xml_diff>
--- a/data_out/teamdata.xlsx
+++ b/data_out/teamdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2223039764837/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="11_C2CE303C21B1A4F5AA873EBF074EE3979B91BC50" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2722993D-989F-4AC1-BE70-2E9584508D30}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_B9923127593964C0B0A62BFA5F3D0198621D4FC7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72B3D179-02DF-4952-B812-0B3BF8C32CF2}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="105">
   <si>
     <t>TeamName</t>
   </si>
@@ -37,6 +37,15 @@
     <t>Devision</t>
   </si>
   <si>
+    <t>ColorCode1</t>
+  </si>
+  <si>
+    <t>ColorCode2</t>
+  </si>
+  <si>
+    <t>ColorCode3</t>
+  </si>
+  <si>
     <t>東京大学</t>
   </si>
   <si>
@@ -49,76 +58,283 @@
     <t>東京六</t>
   </si>
   <si>
+    <t>187FC3</t>
+  </si>
+  <si>
+    <t>F9BE00</t>
+  </si>
+  <si>
     <t>明治大学</t>
   </si>
   <si>
     <t>明治</t>
   </si>
   <si>
+    <t>3E1161</t>
+  </si>
+  <si>
+    <t>FDFCFD</t>
+  </si>
+  <si>
     <t>慶應義塾大学</t>
   </si>
   <si>
     <t>慶應</t>
   </si>
   <si>
+    <t>00256D</t>
+  </si>
+  <si>
+    <t>F60202</t>
+  </si>
+  <si>
+    <t>FFFFFF</t>
+  </si>
+  <si>
     <t>早稲田大学</t>
   </si>
   <si>
     <t>早稲田</t>
   </si>
   <si>
+    <t>61000C</t>
+  </si>
+  <si>
+    <t>F9F4F5</t>
+  </si>
+  <si>
     <t>立教大学</t>
   </si>
   <si>
     <t>立教</t>
   </si>
   <si>
+    <t>000F49</t>
+  </si>
+  <si>
     <t>法政大学</t>
   </si>
   <si>
     <t>法政</t>
   </si>
   <si>
-    <t>61000C</t>
-  </si>
-  <si>
-    <t>00256D</t>
-  </si>
-  <si>
-    <t>3E1161</t>
-  </si>
-  <si>
     <t>FF6400</t>
   </si>
   <si>
-    <t>187FC3</t>
-  </si>
-  <si>
-    <t>000F49</t>
-  </si>
-  <si>
-    <t>ColorCode1</t>
-  </si>
-  <si>
-    <t>ColorCode2</t>
-  </si>
-  <si>
-    <t>ColorCode3</t>
-  </si>
-  <si>
-    <t>F9F4F5</t>
-  </si>
-  <si>
-    <t>F60202</t>
-  </si>
-  <si>
-    <t>FDFCFD</t>
-  </si>
-  <si>
-    <t>FFFFFF</t>
-  </si>
-  <si>
-    <t>F9BE00</t>
+    <t>亜細亜大学</t>
+  </si>
+  <si>
+    <t>亜細亜</t>
+  </si>
+  <si>
+    <t>東都大学野球</t>
+  </si>
+  <si>
+    <t>東都</t>
+  </si>
+  <si>
+    <t>003087</t>
+  </si>
+  <si>
+    <t>C8A400</t>
+  </si>
+  <si>
+    <t>一橋大学</t>
+  </si>
+  <si>
+    <t>一橋</t>
+  </si>
+  <si>
+    <t>004C97</t>
+  </si>
+  <si>
+    <t>学習院大学</t>
+  </si>
+  <si>
+    <t>学習院</t>
+  </si>
+  <si>
+    <t>7A0019</t>
+  </si>
+  <si>
+    <t>駒澤大学</t>
+  </si>
+  <si>
+    <t>駒澤</t>
+  </si>
+  <si>
+    <t>1A2B5C</t>
+  </si>
+  <si>
+    <t>国士舘大学</t>
+  </si>
+  <si>
+    <t>国士舘</t>
+  </si>
+  <si>
+    <t>B51E28</t>
+  </si>
+  <si>
+    <t>芝浦工業大学</t>
+  </si>
+  <si>
+    <t>芝浦工大</t>
+  </si>
+  <si>
+    <t>003366</t>
+  </si>
+  <si>
+    <t>CC0000</t>
+  </si>
+  <si>
+    <t>順天堂大学</t>
+  </si>
+  <si>
+    <t>順天堂</t>
+  </si>
+  <si>
+    <t>007A4B</t>
+  </si>
+  <si>
+    <t>上智大学</t>
+  </si>
+  <si>
+    <t>上智</t>
+  </si>
+  <si>
+    <t>1C5B8A</t>
+  </si>
+  <si>
+    <t>成蹊大学</t>
+  </si>
+  <si>
+    <t>成蹊</t>
+  </si>
+  <si>
+    <t>1A3669</t>
+  </si>
+  <si>
+    <t>D4AF37</t>
+  </si>
+  <si>
+    <t>青山学院大学</t>
+  </si>
+  <si>
+    <t>青山学院</t>
+  </si>
+  <si>
+    <t>00539F</t>
+  </si>
+  <si>
+    <t>C8102E</t>
+  </si>
+  <si>
+    <t>専修大学</t>
+  </si>
+  <si>
+    <t>専修</t>
+  </si>
+  <si>
+    <t>8A0029</t>
+  </si>
+  <si>
+    <t>大正大学</t>
+  </si>
+  <si>
+    <t>大正</t>
+  </si>
+  <si>
+    <t>5C1F69</t>
+  </si>
+  <si>
+    <t>拓殖大学</t>
+  </si>
+  <si>
+    <t>拓殖</t>
+  </si>
+  <si>
+    <t>870017</t>
+  </si>
+  <si>
+    <t>中央大学</t>
+  </si>
+  <si>
+    <t>中央</t>
+  </si>
+  <si>
+    <t>00205B</t>
+  </si>
+  <si>
+    <t>帝京平成大学</t>
+  </si>
+  <si>
+    <t>帝京平成</t>
+  </si>
+  <si>
+    <t>D00027</t>
+  </si>
+  <si>
+    <t>東京科学大学</t>
+  </si>
+  <si>
+    <t>東京科学</t>
+  </si>
+  <si>
+    <t>003F8C</t>
+  </si>
+  <si>
+    <t>東京都市大学</t>
+  </si>
+  <si>
+    <t>東京都市</t>
+  </si>
+  <si>
+    <t>006236</t>
+  </si>
+  <si>
+    <t>東京農業大学</t>
+  </si>
+  <si>
+    <t>東農大</t>
+  </si>
+  <si>
+    <t>1B6B3A</t>
+  </si>
+  <si>
+    <t>B8860B</t>
+  </si>
+  <si>
+    <t>東洋大学</t>
+  </si>
+  <si>
+    <t>東洋</t>
+  </si>
+  <si>
+    <t>002776</t>
+  </si>
+  <si>
+    <t>日本大学</t>
+  </si>
+  <si>
+    <t>BC002D</t>
+  </si>
+  <si>
+    <t>立正大学</t>
+  </si>
+  <si>
+    <t>立正</t>
+  </si>
+  <si>
+    <t>990012</t>
+  </si>
+  <si>
+    <t>國學院大學</t>
+  </si>
+  <si>
+    <t>國學院</t>
+  </si>
+  <si>
+    <t>4B0020</t>
   </si>
 </sst>
 </file>
@@ -154,9 +370,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -453,7 +668,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
@@ -473,136 +688,525 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>27</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="G2" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
       <c r="D3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>21</v>
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>16</v>
       </c>
       <c r="G3" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" t="s">
-        <v>8</v>
-      </c>
       <c r="F4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" t="s">
         <v>20</v>
       </c>
-      <c r="G4" t="s">
-        <v>29</v>
-      </c>
       <c r="H4" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F5" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="G5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F6" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="G6" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" t="s">
         <v>22</v>
       </c>
-      <c r="G7" t="s">
-        <v>31</v>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" t="s">
+        <v>53</v>
+      </c>
+      <c r="G13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" t="s">
+        <v>36</v>
+      </c>
+      <c r="F14" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F15" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" t="s">
+        <v>36</v>
+      </c>
+      <c r="F16" t="s">
+        <v>63</v>
+      </c>
+      <c r="G16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" t="s">
+        <v>36</v>
+      </c>
+      <c r="F17" t="s">
+        <v>67</v>
+      </c>
+      <c r="G17" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>69</v>
+      </c>
+      <c r="B18" t="s">
+        <v>70</v>
+      </c>
+      <c r="C18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" t="s">
+        <v>36</v>
+      </c>
+      <c r="F18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" t="s">
+        <v>36</v>
+      </c>
+      <c r="F19" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" t="s">
+        <v>35</v>
+      </c>
+      <c r="D20" t="s">
+        <v>36</v>
+      </c>
+      <c r="F20" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>78</v>
+      </c>
+      <c r="B21" t="s">
+        <v>79</v>
+      </c>
+      <c r="C21" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21" t="s">
+        <v>36</v>
+      </c>
+      <c r="F21" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" t="s">
+        <v>82</v>
+      </c>
+      <c r="C22" t="s">
+        <v>35</v>
+      </c>
+      <c r="D22" t="s">
+        <v>36</v>
+      </c>
+      <c r="F22" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" t="s">
+        <v>36</v>
+      </c>
+      <c r="F23" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>87</v>
+      </c>
+      <c r="B24" t="s">
+        <v>88</v>
+      </c>
+      <c r="C24" t="s">
+        <v>35</v>
+      </c>
+      <c r="D24" t="s">
+        <v>36</v>
+      </c>
+      <c r="F24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>90</v>
+      </c>
+      <c r="B25" t="s">
+        <v>91</v>
+      </c>
+      <c r="C25" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" t="s">
+        <v>36</v>
+      </c>
+      <c r="F25" t="s">
+        <v>92</v>
+      </c>
+      <c r="G25" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>94</v>
+      </c>
+      <c r="B26" t="s">
+        <v>95</v>
+      </c>
+      <c r="C26" t="s">
+        <v>35</v>
+      </c>
+      <c r="D26" t="s">
+        <v>36</v>
+      </c>
+      <c r="F26" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>97</v>
+      </c>
+      <c r="B27" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D27" t="s">
+        <v>36</v>
+      </c>
+      <c r="F27" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>99</v>
+      </c>
+      <c r="B28" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" t="s">
+        <v>35</v>
+      </c>
+      <c r="D28" t="s">
+        <v>36</v>
+      </c>
+      <c r="F28" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>102</v>
+      </c>
+      <c r="B29" t="s">
+        <v>103</v>
+      </c>
+      <c r="C29" t="s">
+        <v>35</v>
+      </c>
+      <c r="D29" t="s">
+        <v>36</v>
+      </c>
+      <c r="F29" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>